<commit_message>
change sample_subset for EIC
</commit_message>
<xml_diff>
--- a/applications/exercise_study/positive/pos_lipid_reference_set.xlsx
+++ b/applications/exercise_study/positive/pos_lipid_reference_set.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/saralondonoosorio/Documents/GitHub/CEMBIO-EURAC/applications/exercise_study/positive/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCF54DA5-E8C0-CA40-B399-F9DF0D339D4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51CA0B8A-A3D2-904A-A8B9-E03662387F76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4460" yWindow="3960" windowWidth="21360" windowHeight="16780" xr2:uid="{9E5E902E-872A-BE45-A1A9-54571E2C3B45}"/>
+    <workbookView xWindow="4460" yWindow="1140" windowWidth="21360" windowHeight="16780" xr2:uid="{9E5E902E-872A-BE45-A1A9-54571E2C3B45}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="47">
   <si>
     <t>Endogenos</t>
   </si>
@@ -165,6 +165,18 @@
   </si>
   <si>
     <t>cernh4</t>
+  </si>
+  <si>
+    <t>Cer(d40:2)</t>
+  </si>
+  <si>
+    <t>Cer</t>
+  </si>
+  <si>
+    <t>ISTD</t>
+  </si>
+  <si>
+    <t>Sphinganine</t>
   </si>
 </sst>
 </file>
@@ -174,7 +186,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -205,6 +217,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -226,7 +244,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -248,6 +266,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -582,7 +601,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5BFD69E1-DE54-004B-BA8F-573A6CD4FC04}">
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="30.6640625" bestFit="1" customWidth="1"/>
@@ -1062,6 +1081,46 @@
         <v>42</v>
       </c>
     </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A23" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="B23" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="C23" s="11">
+        <v>678.65070000000003</v>
+      </c>
+      <c r="D23" s="11">
+        <v>12</v>
+      </c>
+      <c r="E23" s="11">
+        <v>720</v>
+      </c>
+      <c r="F23" s="11" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A24" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="B24" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="C24" s="11">
+        <v>288.28969999999998</v>
+      </c>
+      <c r="D24" s="11">
+        <v>1.99</v>
+      </c>
+      <c r="E24" s="11">
+        <v>119.4</v>
+      </c>
+      <c r="F24" s="11" t="s">
+        <v>46</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>